<commit_message>
Redesign supervisor dashboard: Process-based cards and detailed monitoring with weekly tracking.
</commit_message>
<xml_diff>
--- a/Newdata/成品入庫TECO狀態.XLSX
+++ b/Newdata/成品入庫TECO狀態.XLSX
@@ -4099,7 +4099,7 @@
         <v>1</v>
       </c>
       <c r="D54" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E54" t="s">
         <v>91</v>
@@ -4117,7 +4117,7 @@
         <v>46134</v>
       </c>
       <c r="J54" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="K54" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Refine supervisor dashboard: compact layout, prioritized finished goods, and include empty processes.
</commit_message>
<xml_diff>
--- a/Newdata/成品入庫TECO狀態.XLSX
+++ b/Newdata/成品入庫TECO狀態.XLSX
@@ -946,6 +946,9 @@
     <t>100003580</t>
   </si>
   <si>
+    <t>REL  PRC  MANC RMWB SETC</t>
+  </si>
+  <si>
     <t>100003585</t>
   </si>
   <si>
@@ -1232,9 +1235,6 @@
   </si>
   <si>
     <t>LG1370NEO機頭P12K,021964_#40,8YU-91,CI</t>
-  </si>
-  <si>
-    <t>REL  PRC  MANC RMWB SETC</t>
   </si>
   <si>
     <t>630000351</t>
@@ -6617,7 +6617,7 @@
         <v>46198</v>
       </c>
       <c r="J104" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="K104" t="s">
         <v>5</v>
@@ -6643,7 +6643,7 @@
         <v>0</v>
       </c>
       <c r="B105" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C105" s="2">
         <v>1</v>
@@ -6682,7 +6682,7 @@
         <v>7</v>
       </c>
       <c r="O105" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="P105" t="s">
         <v>9</v>
@@ -6693,7 +6693,7 @@
         <v>0</v>
       </c>
       <c r="B106" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C106" s="2">
         <v>1</v>
@@ -6732,7 +6732,7 @@
         <v>7</v>
       </c>
       <c r="O106" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="P106" t="s">
         <v>9</v>
@@ -6743,7 +6743,7 @@
         <v>0</v>
       </c>
       <c r="B107" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C107" s="2">
         <v>1</v>
@@ -6767,7 +6767,7 @@
         <v>46253</v>
       </c>
       <c r="J107" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K107" t="s">
         <v>277</v>
@@ -6782,7 +6782,7 @@
         <v>7</v>
       </c>
       <c r="O107" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="P107" t="s">
         <v>9</v>
@@ -6793,7 +6793,7 @@
         <v>0</v>
       </c>
       <c r="B108" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C108" s="2">
         <v>1</v>
@@ -6832,7 +6832,7 @@
         <v>7</v>
       </c>
       <c r="O108" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="P108" t="s">
         <v>9</v>
@@ -6843,7 +6843,7 @@
         <v>0</v>
       </c>
       <c r="B109" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C109" s="2">
         <v>1</v>
@@ -6852,10 +6852,10 @@
         <v>0</v>
       </c>
       <c r="E109" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F109" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G109" s="3">
         <v>46106</v>
@@ -6867,7 +6867,7 @@
         <v>46253</v>
       </c>
       <c r="J109" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K109" t="s">
         <v>277</v>
@@ -6882,7 +6882,7 @@
         <v>7</v>
       </c>
       <c r="O109" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="P109" t="s">
         <v>9</v>
@@ -6893,7 +6893,7 @@
         <v>0</v>
       </c>
       <c r="B110" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C110" s="2">
         <v>1</v>
@@ -6932,7 +6932,7 @@
         <v>7</v>
       </c>
       <c r="O110" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="P110" t="s">
         <v>9</v>
@@ -6943,7 +6943,7 @@
         <v>0</v>
       </c>
       <c r="B111" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C111" s="2">
         <v>1</v>
@@ -6982,7 +6982,7 @@
         <v>7</v>
       </c>
       <c r="O111" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P111" t="s">
         <v>9</v>
@@ -6993,7 +6993,7 @@
         <v>0</v>
       </c>
       <c r="B112" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C112" s="2">
         <v>1</v>
@@ -7017,7 +7017,7 @@
         <v>46190</v>
       </c>
       <c r="J112" t="s">
-        <v>323</v>
+        <v>167</v>
       </c>
       <c r="K112" t="s">
         <v>5</v>
@@ -7032,7 +7032,7 @@
         <v>7</v>
       </c>
       <c r="O112" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P112" t="s">
         <v>9</v>
@@ -7043,7 +7043,7 @@
         <v>0</v>
       </c>
       <c r="B113" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C113" s="2">
         <v>1</v>
@@ -7067,7 +7067,7 @@
         <v>46190</v>
       </c>
       <c r="J113" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K113" t="s">
         <v>5</v>
@@ -7082,7 +7082,7 @@
         <v>7</v>
       </c>
       <c r="O113" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P113" t="s">
         <v>9</v>
@@ -7093,7 +7093,7 @@
         <v>0</v>
       </c>
       <c r="B114" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C114" s="2">
         <v>1</v>
@@ -7117,7 +7117,7 @@
         <v>46254</v>
       </c>
       <c r="J114" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K114" t="s">
         <v>5</v>
@@ -7132,7 +7132,7 @@
         <v>7</v>
       </c>
       <c r="O114" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="P114" t="s">
         <v>9</v>
@@ -7143,7 +7143,7 @@
         <v>0</v>
       </c>
       <c r="B115" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C115" s="2">
         <v>1</v>
@@ -7167,7 +7167,7 @@
         <v>46254</v>
       </c>
       <c r="J115" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K115" t="s">
         <v>5</v>
@@ -7182,7 +7182,7 @@
         <v>7</v>
       </c>
       <c r="O115" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="P115" t="s">
         <v>9</v>
@@ -7193,7 +7193,7 @@
         <v>0</v>
       </c>
       <c r="B116" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C116" s="2">
         <v>1</v>
@@ -7202,10 +7202,10 @@
         <v>0</v>
       </c>
       <c r="E116" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F116" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G116" s="3">
         <v>46113</v>
@@ -7232,7 +7232,7 @@
         <v>7</v>
       </c>
       <c r="O116" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="P116" t="s">
         <v>9</v>
@@ -7243,7 +7243,7 @@
         <v>0</v>
       </c>
       <c r="B117" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C117" s="2">
         <v>1</v>
@@ -7282,7 +7282,7 @@
         <v>7</v>
       </c>
       <c r="O117" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="P117" t="s">
         <v>9</v>
@@ -7293,7 +7293,7 @@
         <v>0</v>
       </c>
       <c r="B118" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C118" s="2">
         <v>1</v>
@@ -7332,7 +7332,7 @@
         <v>7</v>
       </c>
       <c r="O118" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="P118" t="s">
         <v>9</v>
@@ -7343,7 +7343,7 @@
         <v>0</v>
       </c>
       <c r="B119" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C119" s="2">
         <v>1</v>
@@ -7382,7 +7382,7 @@
         <v>7</v>
       </c>
       <c r="O119" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="P119" t="s">
         <v>9</v>
@@ -7393,7 +7393,7 @@
         <v>0</v>
       </c>
       <c r="B120" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C120" s="2">
         <v>1</v>
@@ -7432,7 +7432,7 @@
         <v>7</v>
       </c>
       <c r="O120" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="P120" t="s">
         <v>9</v>
@@ -7443,7 +7443,7 @@
         <v>0</v>
       </c>
       <c r="B121" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C121" s="2">
         <v>1</v>
@@ -7452,10 +7452,10 @@
         <v>0</v>
       </c>
       <c r="E121" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F121" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G121" s="3">
         <v>46122</v>
@@ -7467,7 +7467,7 @@
         <v>46161</v>
       </c>
       <c r="J121" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K121" t="s">
         <v>5</v>
@@ -7482,7 +7482,7 @@
         <v>7</v>
       </c>
       <c r="O121" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="P121" t="s">
         <v>9</v>
@@ -7493,7 +7493,7 @@
         <v>0</v>
       </c>
       <c r="B122" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C122" s="2">
         <v>1</v>
@@ -7532,7 +7532,7 @@
         <v>7</v>
       </c>
       <c r="O122" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="P122" t="s">
         <v>9</v>
@@ -7543,7 +7543,7 @@
         <v>0</v>
       </c>
       <c r="B123" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C123" s="2">
         <v>1</v>
@@ -7567,7 +7567,7 @@
         <v>46168</v>
       </c>
       <c r="J123" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K123" t="s">
         <v>5</v>
@@ -7582,7 +7582,7 @@
         <v>7</v>
       </c>
       <c r="O123" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="P123" t="s">
         <v>9</v>
@@ -7593,7 +7593,7 @@
         <v>0</v>
       </c>
       <c r="B124" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C124" s="2">
         <v>1</v>
@@ -7602,10 +7602,10 @@
         <v>0</v>
       </c>
       <c r="E124" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F124" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G124" s="3">
         <v>46122</v>
@@ -7632,7 +7632,7 @@
         <v>7</v>
       </c>
       <c r="O124" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="P124" t="s">
         <v>9</v>
@@ -7643,7 +7643,7 @@
         <v>0</v>
       </c>
       <c r="B125" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C125" s="2">
         <v>1</v>
@@ -7652,10 +7652,10 @@
         <v>0</v>
       </c>
       <c r="E125" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F125" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G125" s="3">
         <v>46122</v>
@@ -7682,7 +7682,7 @@
         <v>7</v>
       </c>
       <c r="O125" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="P125" t="s">
         <v>9</v>
@@ -7693,7 +7693,7 @@
         <v>0</v>
       </c>
       <c r="B126" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C126" s="2">
         <v>1</v>
@@ -7732,7 +7732,7 @@
         <v>7</v>
       </c>
       <c r="O126" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="P126" t="s">
         <v>9</v>
@@ -7743,7 +7743,7 @@
         <v>0</v>
       </c>
       <c r="B127" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C127" s="2">
         <v>1</v>
@@ -7752,10 +7752,10 @@
         <v>0</v>
       </c>
       <c r="E127" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F127" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G127" s="3">
         <v>46122</v>
@@ -7782,7 +7782,7 @@
         <v>7</v>
       </c>
       <c r="O127" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="P127" t="s">
         <v>9</v>
@@ -7793,7 +7793,7 @@
         <v>0</v>
       </c>
       <c r="B128" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C128" s="2">
         <v>1</v>
@@ -7802,10 +7802,10 @@
         <v>0</v>
       </c>
       <c r="E128" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F128" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G128" s="3">
         <v>46125</v>
@@ -7832,7 +7832,7 @@
         <v>7</v>
       </c>
       <c r="O128" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P128" t="s">
         <v>9</v>
@@ -7843,7 +7843,7 @@
         <v>0</v>
       </c>
       <c r="B129" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C129" s="2">
         <v>1</v>
@@ -7852,10 +7852,10 @@
         <v>0</v>
       </c>
       <c r="E129" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F129" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G129" s="3">
         <v>46125</v>
@@ -7882,7 +7882,7 @@
         <v>7</v>
       </c>
       <c r="O129" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="P129" t="s">
         <v>9</v>
@@ -7893,7 +7893,7 @@
         <v>0</v>
       </c>
       <c r="B130" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C130" s="2">
         <v>1</v>
@@ -7902,10 +7902,10 @@
         <v>0</v>
       </c>
       <c r="E130" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F130" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G130" s="3">
         <v>46126</v>
@@ -7917,7 +7917,7 @@
         <v>46170</v>
       </c>
       <c r="J130" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K130" t="s">
         <v>5</v>
@@ -7932,7 +7932,7 @@
         <v>7</v>
       </c>
       <c r="O130" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="P130" t="s">
         <v>9</v>
@@ -7943,7 +7943,7 @@
         <v>0</v>
       </c>
       <c r="B131" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C131" s="2">
         <v>1</v>
@@ -7952,10 +7952,10 @@
         <v>0</v>
       </c>
       <c r="E131" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F131" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="G131" s="3">
         <v>46127</v>
@@ -7982,7 +7982,7 @@
         <v>7</v>
       </c>
       <c r="O131" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="P131" t="s">
         <v>9</v>
@@ -7993,7 +7993,7 @@
         <v>0</v>
       </c>
       <c r="B132" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C132" s="2">
         <v>1</v>
@@ -8002,10 +8002,10 @@
         <v>0</v>
       </c>
       <c r="E132" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F132" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G132" s="3">
         <v>46132</v>
@@ -8032,7 +8032,7 @@
         <v>7</v>
       </c>
       <c r="O132" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="P132" t="s">
         <v>9</v>
@@ -8043,7 +8043,7 @@
         <v>0</v>
       </c>
       <c r="B133" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C133" s="2">
         <v>1</v>
@@ -8052,10 +8052,10 @@
         <v>0</v>
       </c>
       <c r="E133" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F133" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G133" s="3">
         <v>46133</v>
@@ -8067,7 +8067,7 @@
         <v>46195</v>
       </c>
       <c r="J133" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K133" t="s">
         <v>5</v>
@@ -8082,7 +8082,7 @@
         <v>7</v>
       </c>
       <c r="O133" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="P133" t="s">
         <v>9</v>
@@ -8093,7 +8093,7 @@
         <v>0</v>
       </c>
       <c r="B134" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C134" s="2">
         <v>1</v>
@@ -8102,10 +8102,10 @@
         <v>0</v>
       </c>
       <c r="E134" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F134" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G134" s="3">
         <v>46133</v>
@@ -8117,7 +8117,7 @@
         <v>46195</v>
       </c>
       <c r="J134" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K134" t="s">
         <v>5</v>
@@ -8132,7 +8132,7 @@
         <v>7</v>
       </c>
       <c r="O134" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="P134" t="s">
         <v>9</v>
@@ -8143,7 +8143,7 @@
         <v>0</v>
       </c>
       <c r="B135" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C135" s="2">
         <v>1</v>
@@ -8152,10 +8152,10 @@
         <v>0</v>
       </c>
       <c r="E135" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F135" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G135" s="3">
         <v>46133</v>
@@ -8182,7 +8182,7 @@
         <v>7</v>
       </c>
       <c r="O135" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P135" t="s">
         <v>9</v>
@@ -8193,7 +8193,7 @@
         <v>0</v>
       </c>
       <c r="B136" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C136" s="2">
         <v>1</v>
@@ -8217,7 +8217,7 @@
         <v>46171</v>
       </c>
       <c r="J136" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K136" t="s">
         <v>5</v>
@@ -8232,7 +8232,7 @@
         <v>7</v>
       </c>
       <c r="O136" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="P136" t="s">
         <v>9</v>
@@ -8243,7 +8243,7 @@
         <v>0</v>
       </c>
       <c r="B137" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C137" s="2">
         <v>1</v>
@@ -8252,10 +8252,10 @@
         <v>0</v>
       </c>
       <c r="E137" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F137" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G137" s="3">
         <v>46139</v>
@@ -8282,7 +8282,7 @@
         <v>7</v>
       </c>
       <c r="O137" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="P137" t="s">
         <v>9</v>
@@ -8293,7 +8293,7 @@
         <v>0</v>
       </c>
       <c r="B138" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C138" s="2">
         <v>1</v>
@@ -8332,7 +8332,7 @@
         <v>7</v>
       </c>
       <c r="O138" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="P138" t="s">
         <v>9</v>
@@ -8343,7 +8343,7 @@
         <v>0</v>
       </c>
       <c r="B139" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C139" s="2">
         <v>1</v>
@@ -8382,7 +8382,7 @@
         <v>7</v>
       </c>
       <c r="O139" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="P139" t="s">
         <v>9</v>
@@ -8393,7 +8393,7 @@
         <v>0</v>
       </c>
       <c r="B140" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C140" s="2">
         <v>1</v>
@@ -8432,7 +8432,7 @@
         <v>7</v>
       </c>
       <c r="O140" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="P140" t="s">
         <v>9</v>
@@ -8440,10 +8440,10 @@
     </row>
     <row r="141" spans="1:16">
       <c r="A141" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B141" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C141" s="2">
         <v>1</v>
@@ -8452,10 +8452,10 @@
         <v>0</v>
       </c>
       <c r="E141" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="F141" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="G141" s="3">
         <v>46043</v>
@@ -8470,7 +8470,7 @@
         <v>308</v>
       </c>
       <c r="K141" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="L141" s="3">
         <v>46043</v>
@@ -8479,10 +8479,10 @@
         <v>6</v>
       </c>
       <c r="N141" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="O141" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P141" t="s">
         <v>9</v>
@@ -8490,10 +8490,10 @@
     </row>
     <row r="142" spans="1:16">
       <c r="A142" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B142" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C142" s="2">
         <v>1</v>
@@ -8502,10 +8502,10 @@
         <v>0</v>
       </c>
       <c r="E142" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F142" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="G142" s="3">
         <v>46057</v>
@@ -8520,7 +8520,7 @@
         <v>13</v>
       </c>
       <c r="K142" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="L142" s="3">
         <v>46057</v>
@@ -8529,10 +8529,10 @@
         <v>6</v>
       </c>
       <c r="N142" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="O142" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P142" t="s">
         <v>9</v>
@@ -8540,10 +8540,10 @@
     </row>
     <row r="143" spans="1:16">
       <c r="A143" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B143" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C143" s="2">
         <v>1</v>
@@ -8552,10 +8552,10 @@
         <v>0</v>
       </c>
       <c r="E143" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F143" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="G143" s="3">
         <v>46114</v>
@@ -8567,10 +8567,10 @@
         <v>46148</v>
       </c>
       <c r="J143" t="s">
-        <v>407</v>
+        <v>311</v>
       </c>
       <c r="K143" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="L143" s="3">
         <v>46114</v>
@@ -8579,10 +8579,10 @@
         <v>6</v>
       </c>
       <c r="N143" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="O143" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P143" t="s">
         <v>9</v>
@@ -8590,7 +8590,7 @@
     </row>
     <row r="144" spans="1:16">
       <c r="A144" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B144" t="s">
         <v>408</v>
@@ -8617,10 +8617,10 @@
         <v>46148</v>
       </c>
       <c r="J144" t="s">
-        <v>407</v>
+        <v>311</v>
       </c>
       <c r="K144" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="L144" s="3">
         <v>46122</v>
@@ -8629,10 +8629,10 @@
         <v>6</v>
       </c>
       <c r="N144" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="O144" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P144" t="s">
         <v>9</v>
@@ -8640,7 +8640,7 @@
     </row>
     <row r="145" spans="1:16">
       <c r="A145" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B145" t="s">
         <v>411</v>
@@ -8670,7 +8670,7 @@
         <v>414</v>
       </c>
       <c r="K145" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="L145" s="3">
         <v>46135</v>
@@ -8679,10 +8679,10 @@
         <v>6</v>
       </c>
       <c r="N145" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="O145" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P145" t="s">
         <v>9</v>
@@ -8690,7 +8690,7 @@
     </row>
     <row r="146" spans="1:16">
       <c r="A146" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B146" t="s">
         <v>415</v>
@@ -8720,7 +8720,7 @@
         <v>308</v>
       </c>
       <c r="K146" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="L146" s="3">
         <v>46140</v>
@@ -8729,10 +8729,10 @@
         <v>6</v>
       </c>
       <c r="N146" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="O146" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P146" t="s">
         <v>9</v>

</xml_diff>